<commit_message>
Fix what the develop merge broke; one Jameah refresh at a time
- Job application form (Fathir's update) only sends the lookup lists
  it names; add Student Evaluation Coding, or the academic
  "Appreciation" list is empty and the form cannot be sent (B-42).
- Work telephone extension: a numbers-only field (up to 6 digits) with
  its own check; as a phone-type input the updated form refused "321"
  as an invalid phone number (B-44).
- Jameah academic summary: only one rebuild at a time (database lock);
  a second one is skipped instead of waiting on the table lock, which
  failed a migrate that overlapped the hourly job (B-43). Unit test.
- Browser tests follow the form's steps and its English-letters-only
  name rule.
- Project tracking updated (HR-70, JM-19, B-42 - B-44, TC-REC-13/14).

Tested 22 Oct: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry
views verified, no Error Log entries.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -2722,7 +2722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2772,12 +2772,12 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -2794,17 +2794,17 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -2816,22 +2816,22 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -2848,17 +2848,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -2875,17 +2875,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from Education's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -2897,7 +2897,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -2907,12 +2907,12 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from Education's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -2924,7 +2924,7 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -2934,12 +2934,12 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -2951,25 +2951,52 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="D10" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>

<commit_message>
Test Cases workbook shows the results of the tests/checks scripts
- tests/checks/record.py: each check (files, site, server methods)
  records Pass / Fail and the time (AST) in
  project_tracking/source/automated_results.json; the Test Cases
  builder shows it as the last automated run (TC-ERR-08, TC-ERR-09,
  TC-SEC-10 showed "-" before) (B-52). write_automated_results.py
  keeps these results.
- tests/checks/site.py: import traceback (used when reporting an
  unexpected error); found by tests/checks/files.py (B-53).
- Project tracking updated (B-52, B-53, HR-72, Change Log); all 129
  test cases now show a last automated result.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -2911,7 +2911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2956,17 +2956,17 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Project tracking</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
+          <t>HR-72, B-52, B-53</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
+          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -2978,7 +2978,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -2988,12 +2988,12 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
+          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
+          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -3015,12 +3015,12 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3037,17 +3037,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3059,22 +3059,22 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -3091,17 +3091,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3118,17 +3118,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from Education's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3140,7 +3140,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -3150,12 +3150,12 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from Education's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3167,7 +3167,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
@@ -3177,12 +3177,12 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3194,25 +3194,52 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>

<commit_message>
Add installation and user guides (PDF); count request durations
docs/guides: Installation and Setup Guide (21 pages) and User Guide
(30 pages) for Medical HRMS and Jameah, built from HTML sources with
docs/guides/src/build.py. Screenshots use QA test data only.

Writing the guides found two bugs:
- B-54 Remote Work Request: Duration (Days) was always 0. It is now
  counted on save as working days (calendar days when no holiday list
  covers the dates), and To Date before From Date is refused.
- B-55 Permission Request: Duration (Hours) was always 0 and reversed
  times were accepted. Hours are counted on save and To Time must be
  after From Time.
The patch compute_request_durations fills in saved requests.

Tracking: HR-74, B-54, B-55, TC-ESS-16, CL-37; TC-ESS-02/04 updated.
Re-tested: 95/95 browser checks, 42 unit tests, file/site/API checks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Change Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Checklist'!$A$1:$L$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Checklist'!$A$1:$L$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -684,23 +684,23 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A5)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A5,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A5,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A5,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A5,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -711,23 +711,23 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A6)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A6,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A6,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A6,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A6,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -738,23 +738,23 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A7)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A7,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A7,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A7,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A7,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -765,23 +765,23 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A8)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A8,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A8,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A8,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A8,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -792,23 +792,23 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A9)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A9,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A9,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A9,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A9,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -819,23 +819,23 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$137,$A10)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$138,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A10,Checklist!$H$2:$H$137,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,C$4)</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A10,Checklist!$H$2:$H$137,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,D$4)</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A10,Checklist!$H$2:$H$137,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,E$4)</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$137,$A10,Checklist!$H$2:$H$137,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,F$4)</f>
         <v/>
       </c>
     </row>
@@ -877,7 +877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2900,9 +2900,63 @@
       </c>
       <c r="L37" s="12" t="inlineStr"/>
     </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>CL-37</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>5. Reviews and testing</t>
+        </is>
+      </c>
+      <c r="C38" s="10" t="inlineStr">
+        <is>
+          <t>Share the guides</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>Give HR, managers and the testing team docs/guides/Medical_HRMS_Jameah_User_Guide.pdf, and the server admin docs/guides/Medical_HRMS_Jameah_Installation_Guide.pdf; collect their questions.</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="F38" s="7" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t>HR-74</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K38" s="7" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L38" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L37"/>
-  <conditionalFormatting sqref="H2:H137">
+  <autoFilter ref="A1:L38"/>
+  <conditionalFormatting sqref="H2:H138">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$H2="Open"</formula>
     </cfRule>
@@ -2917,7 +2971,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Open,Done,Blocked,Not needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2931,7 +2985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2976,17 +3030,17 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
+          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
+          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -3008,12 +3062,12 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>HR-72, B-52, B-53</t>
+          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
+          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -3030,17 +3084,17 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Project tracking</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
+          <t>HR-72, B-52, B-53</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
+          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3052,7 +3106,7 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -3062,12 +3116,12 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
+          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
+          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3089,12 +3143,12 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -3111,17 +3165,17 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3133,22 +3187,22 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3165,17 +3219,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3192,17 +3246,17 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3214,7 +3268,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -3224,12 +3278,12 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -3241,7 +3295,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -3251,12 +3305,12 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -3268,25 +3322,52 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>

<commit_message>
Guides and tracker: Academic Presence data sources and open points
User and Installation guides now say where each Academic Presence tab
gets its data, that Proctor Schedules is empty until exam committees
are entered, that Students on Campus counts by hour, and that the
after-4 PM times come from the timetable and class attendance until
attendance devices are connected.

Tracking: HR-37 and HR-38 notes updated, new Checklist CL-38 (enter
exam committees with proctors) and decision DEC-15 (hour slots or the
college's own periods).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Change Log" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Checklist'!$A$1:$L$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Checklist'!$A$1:$L$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -684,23 +684,23 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A5)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F5" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A5,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -711,23 +711,23 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A6)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F6" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A6,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -738,23 +738,23 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A7)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F7" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A7,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -765,23 +765,23 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A8)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F8" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A8,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -792,23 +792,23 @@
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A9)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F9" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A9,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -819,23 +819,23 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Checklist!$B$2:$B$138,$A10)</f>
+        <f>COUNTIF(Checklist!$B$2:$B$139,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,C$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,C$4)</f>
         <v/>
       </c>
       <c r="D10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,D$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,D$4)</f>
         <v/>
       </c>
       <c r="E10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,E$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,E$4)</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>COUNTIFS(Checklist!$B$2:$B$138,$A10,Checklist!$H$2:$H$138,F$4)</f>
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
     </row>
@@ -877,7 +877,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2093,7 +2093,7 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>CL-28</t>
+          <t>CL-38</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
@@ -2103,27 +2103,27 @@
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Leave period for Al Riyada College</t>
+          <t>Exam committees with proctors</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>HR Portal &gt; Leave &gt; Yearly setup 1: Leave Period for this year, company Al Riyada College, tick Is Active.</t>
+          <t>Enter the exam committees (date, time, room) with their proctors; until then Proctor Schedules is empty. Needed to review HR requirement 2.</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>HR</t>
+          <t>Academic Affairs</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Before UAT</t>
+          <t>Before the HR review meeting</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>HR-69</t>
+          <t>HR-37</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
@@ -2134,12 +2134,12 @@
       <c r="I23" s="11" t="inlineStr"/>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr"/>
@@ -2147,7 +2147,7 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>CL-29</t>
+          <t>CL-28</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
@@ -2157,12 +2157,12 @@
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Holiday list for Al Riyada College</t>
+          <t>Leave period for Al Riyada College</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Step 2: Holiday List with the official holidays and weekends; set it as the default holiday list on the Company.</t>
+          <t>HR Portal &gt; Leave &gt; Yearly setup 1: Leave Period for this year, company Al Riyada College, tick Is Active.</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>HR-69, DEC-10</t>
+          <t>HR-69</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -2201,7 +2201,7 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>CL-30</t>
+          <t>CL-29</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Leave approvers</t>
+          <t>Holiday list for Al Riyada College</t>
         </is>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Step 5: set the leave approver on each Department (Leave Approvers table) or on each Employee. Check the Leave setup check on the live server for how many have none.</t>
+          <t>Step 2: Holiday List with the official holidays and weekends; set it as the default holiday list on the Company.</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>HR-69</t>
+          <t>HR-69, DEC-10</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr"/>
@@ -2255,7 +2255,7 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>CL-31</t>
+          <t>CL-30</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
@@ -2265,12 +2265,12 @@
       </c>
       <c r="C26" s="10" t="inlineStr">
         <is>
-          <t>Annual leave balances</t>
+          <t>Leave approvers</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Steps 3-4: submit the annual leave policy (21 or 30 days) and assign it with Leave Control Panel; the Leave setup check turns green.</t>
+          <t>Step 5: set the leave approver on each Department (Leave Approvers table) or on each Employee. Check the Leave setup check on the live server for how many have none.</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="L26" s="12" t="inlineStr"/>
@@ -2309,7 +2309,7 @@
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>CL-32</t>
+          <t>CL-31</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -2319,17 +2319,17 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Sick Leave policy</t>
+          <t>Annual leave balances</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Review and submit 'Medical HRMS - Sick Leave (3 Pay Stages, Separate Sick Year)'; Finance checks the 75% pay on a salary slip.</t>
+          <t>Steps 3-4: submit the annual leave policy (21 or 30 days) and assign it with Leave Control Panel; the Leave setup check turns green.</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>HR + Finance</t>
+          <t>HR</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>HR-20, DEC-14</t>
+          <t>HR-69</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -2363,7 +2363,7 @@
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>CL-22</t>
+          <t>CL-32</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -2373,27 +2373,27 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Attendance devices</t>
+          <t>Sick Leave policy</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Connect the devices so Faculty After 4 PM uses real check-out times.</t>
+          <t>Review and submit 'Medical HRMS - Sick Leave (3 Pay Stages, Separate Sick Year)'; Finance checks the 75% pay on a salary slip.</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>HR + IT</t>
+          <t>HR + Finance</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Later</t>
+          <t>Before UAT</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>HR-56</t>
+          <t>HR-20, DEC-14</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2404,12 +2404,12 @@
       <c r="I28" s="11" t="inlineStr"/>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="K28" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="L28" s="12" t="inlineStr"/>
@@ -2417,37 +2417,37 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>CL-23</t>
+          <t>CL-22</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>5. Reviews and testing</t>
+          <t>4. HR data</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Run the test cases</t>
+          <t>Attendance devices</t>
         </is>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Testing team works through Medical_HRMS_Jameah_Test_Cases.xlsx and records results and bugs there.</t>
+          <t>Connect the devices so Faculty After 4 PM uses real check-out times.</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Testing team</t>
+          <t>HR + IT</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>HR-46</t>
+          <t>HR-56</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
@@ -2471,7 +2471,7 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>CL-24</t>
+          <t>CL-23</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -2481,17 +2481,17 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Arabic labels</t>
+          <t>Run the test cases</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>An Arabic speaker reads the HR / Employee Portal pages in Arabic and lists wording to change, including the 114 new leave texts (22 Oct).</t>
+          <t>Testing team works through Medical_HRMS_Jameah_Test_Cases.xlsx and records results and bugs there.</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Project owner</t>
+          <t>Testing team</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -2501,7 +2501,7 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>HR-66, HR-68</t>
+          <t>HR-46</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="L30" s="12" t="inlineStr"/>
@@ -2525,7 +2525,7 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>CL-25</t>
+          <t>CL-24</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -2535,12 +2535,12 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Portal design approval</t>
+          <t>Arabic labels</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Client confirms the new HR Portal / Employee Portal look.</t>
+          <t>An Arabic speaker reads the HR / Employee Portal pages in Arabic and lists wording to change, including the 114 new leave texts (22 Oct).</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-66, HR-68</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="K31" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="L31" s="12" t="inlineStr"/>
@@ -2579,7 +2579,7 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>CL-33</t>
+          <t>CL-25</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -2589,17 +2589,17 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Leave flow UAT</t>
+          <t>Portal design approval</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>An employee and their manager go through TC-LV-09 - TC-LV-17: plan, apply now, approve, return (also after sick leave).</t>
+          <t>Client confirms the new HR Portal / Employee Portal look.</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Testing team</t>
+          <t>Project owner</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>HR-68</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2620,12 +2620,12 @@
       <c r="I32" s="11" t="inlineStr"/>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="K32" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="L32" s="12" t="inlineStr"/>
@@ -2633,7 +2633,7 @@
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>CL-26</t>
+          <t>CL-33</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -2643,12 +2643,12 @@
       </c>
       <c r="C33" s="10" t="inlineStr">
         <is>
-          <t>Arabic interface</t>
+          <t>Leave flow UAT</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>Switch to AR and repeat a few test cases (HR Portal, Employee Portal, application form).</t>
+          <t>An employee and their manager go through TC-LV-09 - TC-LV-17: plan, apply now, approve, return (also after sick leave).</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2663,7 +2663,7 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>HR-68</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
@@ -2674,12 +2674,12 @@
       <c r="I33" s="11" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="K33" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="L33" s="12" t="inlineStr"/>
@@ -2687,7 +2687,7 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>CL-27</t>
+          <t>CL-26</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -2697,22 +2697,22 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Developer copy of the education app up to date</t>
+          <t>Arabic interface</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
-          <t>On the development machine the education app checkout is behind its master branch; update it before testing there (git pull --ff-only).</t>
+          <t>Switch to AR and repeat a few test cases (HR Portal, Employee Portal, application form).</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Project owner</t>
+          <t>Testing team</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Now</t>
+          <t>UAT</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="K34" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="L34" s="12" t="inlineStr"/>
@@ -2741,22 +2741,22 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>CL-34</t>
+          <t>CL-27</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>6. Team and repository</t>
+          <t>5. Reviews and testing</t>
         </is>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>Delete the merged branches on GitHub</t>
+          <t>Developer copy of the education app up to date</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
         <is>
-          <t>After UAT: feature/uat-2026-10-22, feature/hr-portal-design, feature/jameah-ministry-views, fix/hrm-e2e-approval-permission-bugs, ministry-lookup, employee-applicant (all merged into develop; their history stays in develop).</t>
+          <t>On the development machine the education app checkout is behind its master branch; update it before testing there (git pull --ff-only).</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>After UAT</t>
+          <t>Now</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>HR-71</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H35" s="11" t="inlineStr">
@@ -2782,7 +2782,7 @@
       <c r="I35" s="11" t="inlineStr"/>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="K35" s="7" t="inlineStr">
@@ -2795,7 +2795,7 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>CL-35</t>
+          <t>CL-34</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -2805,12 +2805,12 @@
       </c>
       <c r="C36" s="10" t="inlineStr">
         <is>
-          <t>Assign the open tasks</t>
+          <t>Delete the merged branches on GitHub</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
         <is>
-          <t>Task Tracker, Tasks sheet: pick who each open task is given to in the Assigned to column (dropdown; e.g. HR-73, HR-16, HR-17, HR-25, JM-15, JM-19).</t>
+          <t>After UAT: feature/uat-2026-10-22, feature/hr-portal-design, feature/jameah-ministry-views, fix/hrm-e2e-approval-permission-bugs, ministry-lookup, employee-applicant (all merged into develop; their history stays in develop).</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -2820,12 +2820,12 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Now</t>
+          <t>After UAT</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
         <is>
-          <t>HR-73</t>
+          <t>HR-71</t>
         </is>
       </c>
       <c r="H36" s="11" t="inlineStr">
@@ -2849,7 +2849,7 @@
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>CL-36</t>
+          <t>CL-35</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -2859,27 +2859,27 @@
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Checks before every release</t>
+          <t>Assign the open tasks</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>python3 tests/checks/files.py; fx.py tests/checks/site.py; python3 tests/checks/api_methods.py; then the browser suite (tests/e2e/README.md). All must pass.</t>
+          <t>Task Tracker, Tasks sheet: pick who each open task is given to in the Assigned to column (dropdown; e.g. HR-73, HR-16, HR-17, HR-25, JM-15, JM-19).</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Developer (Abdul Hakeem)</t>
+          <t>Project owner</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Every release</t>
+          <t>Now</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>HR-72</t>
+          <t>HR-73</t>
         </is>
       </c>
       <c r="H37" s="11" t="inlineStr">
@@ -2903,37 +2903,37 @@
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>CL-37</t>
+          <t>CL-36</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>5. Reviews and testing</t>
+          <t>6. Team and repository</t>
         </is>
       </c>
       <c r="C38" s="10" t="inlineStr">
         <is>
-          <t>Share the guides</t>
+          <t>Checks before every release</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Give HR, managers and the testing team docs/guides/Medical_HRMS_Jameah_User_Guide.pdf, and the server admin docs/guides/Medical_HRMS_Jameah_Installation_Guide.pdf; collect their questions.</t>
+          <t>python3 tests/checks/files.py; fx.py tests/checks/site.py; python3 tests/checks/api_methods.py; then the browser suite (tests/e2e/README.md). All must pass.</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Project owner</t>
+          <t>Developer (Abdul Hakeem)</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>UAT</t>
+          <t>Every release</t>
         </is>
       </c>
       <c r="G38" s="7" t="inlineStr">
         <is>
-          <t>HR-74</t>
+          <t>HR-72</t>
         </is>
       </c>
       <c r="H38" s="11" t="inlineStr">
@@ -2954,9 +2954,63 @@
       </c>
       <c r="L38" s="12" t="inlineStr"/>
     </row>
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>CL-37</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>5. Reviews and testing</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>Share the guides</t>
+        </is>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Give HR, managers and the testing team docs/guides/Medical_HRMS_Jameah_User_Guide.pdf, and the server admin docs/guides/Medical_HRMS_Jameah_Installation_Guide.pdf; collect their questions.</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Project owner</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>UAT</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>HR-74</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K39" s="7" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L38"/>
-  <conditionalFormatting sqref="H2:H138">
+  <autoFilter ref="A1:L39"/>
+  <conditionalFormatting sqref="H2:H139">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
       <formula>$H2="Open"</formula>
     </cfRule>
@@ -2971,7 +3025,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Open,Done,Blocked,Not needed"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2985,7 +3039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3035,12 +3089,12 @@
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
+          <t>HR-37, HR-38, DEC-15, CL-38</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
+          <t>Academic Presence (HR requirements 1-4) checked against the client's request: all four are on the HR Dashboard and tested. The guides now say where each tab's data comes from, that Proctor Schedules stays empty until exam committees are entered (new Checklist CL-38), that Students on Campus counts by hour, and that after-4 PM times come from the timetable and class attendance until devices are connected. New decision DEC-15: hour slots or the college's own periods.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -3057,17 +3111,17 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
+          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
+          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -3089,12 +3143,12 @@
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>HR-72, B-52, B-53</t>
+          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
+          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3111,17 +3165,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Project tracking</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
+          <t>HR-72, B-52, B-53</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
+          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3133,7 +3187,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
@@ -3143,12 +3197,12 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
+          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
+          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -3170,12 +3224,12 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3192,17 +3246,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3214,22 +3268,22 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3246,17 +3300,17 @@
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3273,17 +3327,17 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -3295,7 +3349,7 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
@@ -3305,12 +3359,12 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -3322,7 +3376,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -3332,12 +3386,12 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3349,25 +3403,52 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C14" s="10" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D14" s="10" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>

<commit_message>
Tracking: testing team UAT round started (27 Oct)
Test Cases workbook and both PDF guides handed to the testing team.
New task HR-75 (In progress, assigned to the testing team); Checklist
CL-23 and CL-37 In progress, with a new blue "In progress" status.
Checklist summary now shows every status column (Not needed was cut).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -146,7 +146,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <font>
         <b val="1"/>
@@ -156,6 +156,18 @@
         <patternFill patternType="solid">
           <fgColor rgb="00EF6C00"/>
           <bgColor rgb="00EF6C00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="001565C0"/>
+          <bgColor rgb="001565C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -574,7 +586,7 @@
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Al-Riyada College for Health Sciences · last updated 23 Oct 2026</t>
+          <t>Al-Riyada College for Health Sciences · last updated 27 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -620,15 +632,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -663,15 +676,20 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Blocked</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Not needed</t>
         </is>
@@ -703,6 +721,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G5" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A5,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -730,6 +752,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G6" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A6,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
@@ -757,6 +783,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G7" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A7,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
@@ -784,6 +814,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G8" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A8,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
@@ -811,6 +845,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G9" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A9,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
@@ -838,6 +876,10 @@
         <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,F$4)</f>
         <v/>
       </c>
+      <c r="G10" s="7">
+        <f>COUNTIFS(Checklist!$B$2:$B$139,$A10,Checklist!$H$2:$H$139,G$4)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -863,6 +905,10 @@
       </c>
       <c r="F11" s="8">
         <f>SUM(F5:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="8">
+        <f>SUM(G5:G10)</f>
         <v/>
       </c>
     </row>
@@ -2486,7 +2532,7 @@
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Testing team works through Medical_HRMS_Jameah_Test_Cases.xlsx and records results and bugs there.</t>
+          <t>Testing team works through Medical_HRMS_Jameah_Test_Cases.xlsx and records results and bugs there. Started 27 Oct with the test cases and both guides.</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2501,12 +2547,12 @@
       </c>
       <c r="G30" s="7" t="inlineStr">
         <is>
-          <t>HR-46</t>
+          <t>HR-46, HR-75</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I30" s="11" t="inlineStr"/>
@@ -2517,7 +2563,7 @@
       </c>
       <c r="K30" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>27 Oct 2026</t>
         </is>
       </c>
       <c r="L30" s="12" t="inlineStr"/>
@@ -2972,7 +3018,7 @@
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Give HR, managers and the testing team docs/guides/Medical_HRMS_Jameah_User_Guide.pdf, and the server admin docs/guides/Medical_HRMS_Jameah_Installation_Guide.pdf; collect their questions.</t>
+          <t>Give HR, managers and the testing team docs/guides/Medical_HRMS_Jameah_User_Guide.pdf, and the server admin docs/guides/Medical_HRMS_Jameah_Installation_Guide.pdf; collect their questions. 27 Oct: given to the testing team; still to give to HR, managers and the server admin.</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -2987,12 +3033,12 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>HR-74</t>
+          <t>HR-74, HR-75</t>
         </is>
       </c>
       <c r="H39" s="11" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I39" s="11" t="inlineStr"/>
@@ -3003,7 +3049,7 @@
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>27 Oct 2026</t>
         </is>
       </c>
       <c r="L39" s="12" t="inlineStr"/>
@@ -3015,18 +3061,21 @@
       <formula>$H2="Open"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
+      <formula>$H2="In progress"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
       <formula>$H2="Done"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
+    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
       <formula>$H2="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" dxfId="3" stopIfTrue="1">
+    <cfRule type="expression" priority="5" dxfId="4" stopIfTrue="1">
       <formula>$H2="Not needed"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation sqref="H2:H139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Open,Done,Blocked,Not needed"</formula1>
+      <formula1>"Open,In progress,Done,Blocked,Not needed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3039,7 +3088,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3079,22 +3128,22 @@
     <row r="2">
       <c r="A2" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>27 Oct 2026</t>
         </is>
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>HR-37, HR-38, DEC-15, CL-38</t>
+          <t>HR-75, CL-23, CL-37</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Academic Presence (HR requirements 1-4) checked against the client's request: all four are on the HR Dashboard and tested. The guides now say where each tab's data comes from, that Proctor Schedules stays empty until exam committees are entered (new Checklist CL-38), that Students on Campus counts by hour, and that after-4 PM times come from the timetable and class attendance until devices are connected. New decision DEC-15: hour slots or the college's own periods.</t>
+          <t>Test Cases workbook and both PDF guides given to the testing team; their UAT round has started (HR-75 In progress). Checklist: new status 'In progress' (blue); CL-23 Run the test cases and CL-37 Share the guides are In progress (the guides still go to HR, managers and the server admin). Testing team added to the Assigned to list.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -3116,12 +3165,12 @@
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
+          <t>HR-37, HR-38, DEC-15, CL-38</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
+          <t>Academic Presence (HR requirements 1-4) checked against the client's request: all four are on the HR Dashboard and tested. The guides now say where each tab's data comes from, that Proctor Schedules stays empty until exam committees are entered (new Checklist CL-38), that Students on Campus counts by hour, and that after-4 PM times come from the timetable and class attendance until devices are connected. New decision DEC-15: hour slots or the college's own periods.</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -3138,17 +3187,17 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
+          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
+          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3170,12 +3219,12 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-72, B-52, B-53</t>
+          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
+          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3192,17 +3241,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Project tracking</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
+          <t>HR-72, B-52, B-53</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
+          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -3214,7 +3263,7 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -3224,12 +3273,12 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
+          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
+          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3251,12 +3300,12 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3273,17 +3322,17 @@
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3295,22 +3344,22 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3327,17 +3376,17 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -3354,17 +3403,17 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -3376,7 +3425,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -3386,12 +3435,12 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3403,7 +3452,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -3413,12 +3462,12 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -3430,25 +3479,52 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C15" s="10" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>

<commit_message>
QA cleanup: stop unsent QA e-mails instead of deleting them
The e-mail job could be sending them while they were deleted and logged
'Email Queue ... not found'.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
+++ b/project_tracking/Medical_HRMS_Jameah_Checklist.xlsx
@@ -3250,7 +3250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>Round 2</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C2" s="10" t="inlineStr">
         <is>
-          <t>HR-16, HR-24, HR-25, HR-48, HR-76, HR-77, B-26, B-56, B-57, DEC-16, CL-39 - CL-41, TC-APR-02, TC-APR-09 - TC-APR-13, TC-ESS-17 - TC-ESS-23, TC-EMP-13, TC-EMP-14, TC-LV-18</t>
+          <t>HR-76</t>
         </is>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>Round 2: employees change, send or delete their drafts and send a rejected request again; rejecting needs a reason, which the employee reads with the request's history; notifications in the bell (and e-mail where the mail account works) for HR on new requests and for the employee at every later step; the Instructor and Academic Advisor forms save after an Employee is picked (B-26, B-56); amounts say SAR; the bell shows the time as text (B-57). New: Round column in the Test Cases workbook, the Round 2 document for the testers, User Guide and Installation Guide updated. Re-tested: 101/101 browser checks, 52 unit tests (0 failures), 0 file and 0 site problems, 31 server methods x 3 roles; Error Log: only the known e-mail password error B-25 (notification e-mails this copy cannot send).</t>
+          <t>QA cleanup stops the unsent e-mails of removed QA records (status Error) instead of deleting them: the e-mail job could be sending them at that moment and logged 'Email Queue ... not found'.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -3322,17 +3322,17 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Round 2</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
         <is>
-          <t>HR-75, CL-23, CL-37</t>
+          <t>HR-16, HR-24, HR-25, HR-48, HR-76, HR-77, B-26, B-56, B-57, DEC-16, CL-39 - CL-41, TC-APR-02, TC-APR-09 - TC-APR-13, TC-ESS-17 - TC-ESS-23, TC-EMP-13, TC-EMP-14, TC-LV-18</t>
         </is>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Test Cases workbook and both PDF guides given to the testing team; their UAT round has started (HR-75 In progress). Checklist: new status 'In progress' (blue); CL-23 Run the test cases and CL-37 Share the guides are In progress (the guides still go to HR, managers and the server admin). Testing team added to the Assigned to list.</t>
+          <t>Round 2: employees change, send or delete their drafts and send a rejected request again; rejecting needs a reason, which the employee reads with the request's history; notifications in the bell (and e-mail where the mail account works) for HR on new requests and for the employee at every later step; the Instructor and Academic Advisor forms save after an Employee is picked (B-26, B-56); amounts say SAR; the bell shows the time as text (B-57). New: Round column in the Test Cases workbook, the Round 2 document for the testers, User Guide and Installation Guide updated. Re-tested: 101/101 browser checks, 52 unit tests (0 failures), 0 file and 0 site problems, 31 server methods x 3 roles; Error Log: only the known e-mail password error B-25 (notification e-mails this copy cannot send).</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -3344,22 +3344,22 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>23 Oct 2026</t>
+          <t>27 Oct 2026</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
         <is>
-          <t>HR-37, HR-38, DEC-15, CL-38</t>
+          <t>HR-75, CL-23, CL-37</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>Academic Presence (HR requirements 1-4) checked against the client's request: all four are on the HR Dashboard and tested. The guides now say where each tab's data comes from, that Proctor Schedules stays empty until exam committees are entered (new Checklist CL-38), that Students on Campus counts by hour, and that after-4 PM times come from the timetable and class attendance until devices are connected. New decision DEC-15: hour slots or the college's own periods.</t>
+          <t>Test Cases workbook and both PDF guides given to the testing team; their UAT round has started (HR-75 In progress). Checklist: new status 'In progress' (blue); CL-23 Run the test cases and CL-37 Share the guides are In progress (the guides still go to HR, managers and the server admin). Testing team added to the Assigned to list.</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -3381,12 +3381,12 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
+          <t>HR-37, HR-38, DEC-15, CL-38</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
+          <t>Academic Presence (HR requirements 1-4) checked against the client's request: all four are on the HR Dashboard and tested. The guides now say where each tab's data comes from, that Proctor Schedules stays empty until exam committees are entered (new Checklist CL-38), that Students on Campus counts by hour, and that after-4 PM times come from the timetable and class attendance until devices are connected. New decision DEC-15: hour slots or the college's own periods.</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -3403,17 +3403,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Project tracking</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
+          <t>HR-74, B-54, B-55, TC-ESS-02, TC-ESS-04, TC-ESS-16, CL-37</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
+          <t>Installation and Setup Guide (21 pages) and User Guide (30 pages) in PDF, with screenshots from the test site (QA data only); sources in docs/guides/src. Fixed while writing them: Remote Work Request duration and Permission Request hours were always 0 (now counted; reversed times refused; a patch fills in saved requests). Re-tested: 95/95 browser checks, 42 unit tests (0 failures), 0 file and 0 site problems, 29 server methods x 3 roles, no Error Log entries.</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -3435,12 +3435,12 @@
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>HR-72, B-52, B-53</t>
+          <t>All tasks; HR-04 - HR-06, HR-11, HR-12, HR-28 - HR-30, HR-48, HR-66, HR-70, HR-71, HR-73, JM-03, JM-06, JM-12, JM-13, JM-16, JM-17, B-26, B-34, CL-35</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
+          <t>Owners corrected: Abdul Hakeem designed and built Medical HRMS and Jameah and leads every development task. New column 'Assigned to' (with a dropdown) shows who a task was given to: Dinesh (HR-06, and HR-04 at first), Fathir (HR-04, HR-05, HR-70), otherwise Abdul Hakeem; client-side tasks stay with HR, Academic Affairs, the Registrar or the server admin. Wording that credited others for this work removed. Status and Priority shown in clear colours in all three workbooks (Status, Priority, Result and Severity cells only), with a priority legend in the Read Me.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -3457,17 +3457,17 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Project tracking</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
+          <t>HR-72, B-52, B-53</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
+          <t>The three check scripts (files, site, server methods) now record their result in the Test Cases workbook (Last automated run: Pass, 23 Oct). The file check found a missing import in the site check; fixed.</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -3479,7 +3479,7 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>22 Oct 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -3489,12 +3489,12 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
+          <t>HR-58, HR-69, HR-71 - HR-73, B-45 - B-51, CL-01, CL-30, CL-34 - CL-36, TC-ERR-06 - TC-ERR-09, TC-SEC-10</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
+          <t>Every branch merged into develop (ministry-lookup last; employee-applicant recorded as merged without its July files, as decided); develop is now the branch to test and deploy. Full check of every file and page (files, site, server methods by role, unit tests, browser suite with a sweep of every Medical HRMS doctype); checks kept in tests/checks. Fixed: stray files, outdated README and developer guide, QA setup race, refresh-lock test, Ministry code search. HR-69 corrected (employee counts were test hires). Result: 95/95 browser checks (error sweep: 116 pages for HR, 20 for employees), 37/37 unit tests, 23/23 Ministry views, 29 server methods x 3 roles, 0 file and 0 site problems, no Error Log entries.</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -3516,12 +3516,12 @@
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
+          <t>HR-58, HR-70, JM-05, JM-19, B-42 – B-44, TC-REC-13, TC-REC-14</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
+          <t>develop (Fathir's job application update, PR #2) merged into feature/uat-2026-10-22; conflicts in job_application.py, job-application.html and ar.csv resolved keeping both sides; the Appreciation list restored and the work extension accepted again on the updated form (B-42, B-44); a migrate no longer fails when it overlaps the hourly Jameah refresh (B-43); test output removed from the repository. Re-tested: 95/95 browser checks, 37/37 unit tests, 23/23 Ministry views OK, no Error Log entries. Branch to test and deploy: feature/uat-2026-10-22.</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -3538,17 +3538,17 @@
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Testing</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>HR-67, B-41</t>
+          <t>HR-08, HR-09, HR-19, HR-20, HR-22, HR-68, HR-69, B-36 – B-40, DEC-14, CL-28 – CL-33</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
+          <t>Leave made one flow: Leave Plan (employees send it; manager and department head approve) -&gt; Leave Application (only leave the employee holds, with the days left; Apply now from an approved plan) -&gt; Leave Return (asked for when a leave ends; certificate and occupational health only after sick leave). Sick-leave types renamed in pay order (Sick Leave 1 / 2 / 3) by a migration patch. HR Portal Leave section: setup check per company, daily leave counts, yearly setup in order. Arabic for 114 new texts. 5 unit tests and 7 browser tests (LV-01 - LV-07); test cases TC-LV-09 - 17, TC-HRD-06/07. Real company Al Riyada College still needs its leave setup (HR-69). Branch to test and deploy: feature/uat-2026-10-22 (all work to date).</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -3560,22 +3560,22 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>21 Oct 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Testing</t>
         </is>
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
+          <t>HR-67, B-41</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
+          <t>Browser test suite, QA data scripts and the results helper kept in the repository (tests/e2e); the QA scripts only run on a site named in QA_TEST_SITE. The QA reset no longer leaves the QA HR User without access to its own My Settings (test data only). The leave unit test now attaches a real test file, so it no longer writes 'Error Attaching File' to the Error Log. Full run 22 Oct: 95/95 browser checks, 36/36 unit tests, 23/23 Ministry views OK, no new Error Log entries.</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -3592,17 +3592,17 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS</t>
+          <t>Medical HRMS + Jameah</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>HR-66</t>
+          <t>HR-49, HR-50, HR-51, HR-65, JM-14, B-35, DEC-12, DEC-13</t>
         </is>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
+          <t>Report 'Employees Missing Ministry Data'; data sheet for non-academic staff (download, check, import); unused duplicate applicant Ministry fields removed; Create Employee dialog asks for every field the Employee form requires; Jameah Faculty views (8) built and verified (23 views in all). Arabic for the 46 new labels. Documents moved to the project_tracking folder; Checklist workbook added; dates on every row; HRM_TASK_TRACKER.md marked as superseded.</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -3619,17 +3619,17 @@
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Medical HRMS + Jameah</t>
+          <t>Medical HRMS</t>
         </is>
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
+          <t>HR-66</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
+          <t>HR Portal and Employee Portal in the new college portal design (menu, top bar, EN/AR, dark mode); Arabic translations for these pages.</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -3641,7 +3641,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>20 Oct 2026</t>
+          <t>21 Oct 2026</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -3651,12 +3651,12 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
+          <t>HR-12, HR-31, HR-32, HR-45, HR-46, HR-59 – HR-64, JM-17, JM-18, B-24 – B-34</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
+          <t>End-to-end test round 3 with an error sweep of every page: fixes for the errors the client reported (non-Saudi employees, breadcrumb 'Not permitted', Cost Center pop-up, academic hire e-mail, Holiday List); HR login lands on the HR Dashboard; Ministry GPA and credit hours from the college's official calculation. Test Report, Test Cases and Task Tracker created.</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -3668,7 +3668,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>19 Oct 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -3678,12 +3678,12 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+          <t>HR-07 – HR-09, HR-13 – HR-15, HR-19, HR-22, HR-26, HR-36 – HR-44, JM-02 – JM-07, B-12 – B-23</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+          <t>Jameah Employee (5) and Student (10) views built and verified value by value; Academic Presence; browser test round 2 fixes.</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -3695,25 +3695,52 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
+          <t>19 Oct 2026</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Medical HRMS + Jameah</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>HR-02, HR-05, HR-06, HR-24, HR-27, HR-33 – HR-35, JM-01, B-01 – B-11</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Browser end-to-end test round 1 and fixes (approvals, recruitment security, Ministry identity rules); Instructor data sheet; Jameah research.</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Abdul Hakeem</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
           <t>1 Oct 2026</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Medical HRMS</t>
         </is>
       </c>
-      <c r="C17" s="10" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>HR-01 – HR-32</t>
         </is>
       </c>
-      <c r="D17" s="10" t="inlineStr">
+      <c r="D18" s="10" t="inlineStr">
         <is>
           <t>First HRM task tracker (HRM_TASK_TRACKER.md / .csv).</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>Team</t>
         </is>

</xml_diff>